<commit_message>
O8 lock-screen privacy per category; O9 traceability for feature tests
O8: lock-screen text is neutral for worship, health, money and third-party
items by default. More > Lock-screen details lets the user show details per
category. Neutral text en/bn, Mix derived from bn. ROADMAP O8 marked built in
code; on-device lock-screen check stays Owner-only.

O9: traceability.json now maps the feature test files whose assertions match a
TM-TST criterion (10 new rows, 2 extended). Files that do not fit are listed
in docs/register/EVIDENCE_REFRESH.md under "Not yet mapped" with the reason.
Register evidence copy regenerated from the unchanged v2.0 file.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQLEnTuJEEpTPr8wz4yQ9
</commit_message>
<xml_diff>
--- a/docs/register/Trillionaire_Me_Requirements_Register_v2_1_evidence_refresh.xlsx
+++ b/docs/register/Trillionaire_Me_Requirements_Register_v2_1_evidence_refresh.xlsx
@@ -5246,7 +5246,7 @@
       </c>
       <c r="O44" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="O46" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -6078,7 +6078,7 @@
       </c>
       <c r="O56" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -8569,7 +8569,7 @@
       </c>
       <c r="O91" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -10577,7 +10577,7 @@
       </c>
       <c r="O119" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -10646,7 +10646,7 @@
       </c>
       <c r="O120" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="O149" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -12817,7 +12817,7 @@
       </c>
       <c r="O151" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -13024,7 +13024,7 @@
       </c>
       <c r="O154" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -13304,7 +13304,7 @@
       </c>
       <c r="O158" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -13515,7 +13515,7 @@
       </c>
       <c r="O161" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -14006,7 +14006,7 @@
       </c>
       <c r="O168" s="14" t="inlineStr">
         <is>
-          <t>Not verified — no build</t>
+          <t>Partial — automated part passes; manual/human gate pending — see Tests v2</t>
         </is>
       </c>
     </row>
@@ -15976,12 +15976,12 @@
       <c r="H24" s="14" t="n"/>
       <c r="I24" s="14" t="inlineStr">
         <is>
-          <t>Pass (G1) — G1 automated: 1000-case property test + browser e2e (blank and 'don't know' never stored as 0)</t>
+          <t>Pass (G1) — G1 automated: 1000-case property test + browser e2e (blank and 'don't know' never stored as 0); goal form blank horizon and B9 plan blank inputs stay unset, never 0 (unit)</t>
         </is>
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>tests/g1.test.ts; tools/e2e.mjs; evidence/e2e-report.json</t>
+          <t>tests/g1.test.ts; tools/e2e.mjs; evidence/e2e-report.json; tests/goal_form.test.ts; tests/b9_plan_flow.test.ts</t>
         </is>
       </c>
       <c r="K24" s="14" t="n"/>
@@ -16896,10 +16896,14 @@
       <c r="H44" s="14" t="n"/>
       <c r="I44" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J44" s="14" t="n"/>
+          <t>Partial (G1) — Copy string scan: no banned punitive/judging words in en, bn or mix across all keys (habit-specific wording in TM-TST-148). Review of copy by a human not done</t>
+        </is>
+      </c>
+      <c r="J44" s="14" t="inlineStr">
+        <is>
+          <t>tests/copy_review.test.ts</t>
+        </is>
+      </c>
       <c r="K44" s="14" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="10">
@@ -16986,10 +16990,14 @@
       <c r="H46" s="14" t="n"/>
       <c r="I46" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J46" s="14" t="n"/>
+          <t>Partial (G1) — O6 90-day review: no records gives 'not enough data' (null, never 0); only in-window records counted. Weekly review itself not covered</t>
+        </is>
+      </c>
+      <c r="J46" s="14" t="inlineStr">
+        <is>
+          <t>tests/o6_reality_review_templates.test.ts</t>
+        </is>
+      </c>
       <c r="K46" s="14" t="n"/>
     </row>
     <row r="47" ht="21.75" customHeight="1" s="10">
@@ -17436,10 +17444,14 @@
       <c r="H56" s="14" t="n"/>
       <c r="I56" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J56" s="14" t="n"/>
+          <t>Partial (G1) — O7 own options + saved offline search list: save, cap 20 per field, add-own, source snapshot kept for offline reuse, secrets refused. Select/compare/customize/reject/defer and replace-history not covered</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="inlineStr">
+        <is>
+          <t>tests/o7_own_saved_lists.test.ts</t>
+        </is>
+      </c>
       <c r="K56" s="14" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="10">
@@ -19087,10 +19099,14 @@
       </c>
       <c r="I91" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J91" s="14" t="n"/>
+          <t>Partial (G1) — G2 backup/restore round-trip into a clean database; damaged or tampered file rejected; demo backup never restored as real; newer schema refused. Device-level checksum and attachments not covered</t>
+        </is>
+      </c>
+      <c r="J91" s="14" t="inlineStr">
+        <is>
+          <t>tests/g2.test.ts</t>
+        </is>
+      </c>
       <c r="K91" s="14" t="n"/>
     </row>
     <row r="92" ht="21.75" customHeight="1" s="10">
@@ -20415,10 +20431,14 @@
       <c r="H119" s="14" t="n"/>
       <c r="I119" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J119" s="14" t="n"/>
+          <t>Partial (G1) — Calm copy guard on the stuck and log keys: no judging, score, streak or grade words in en/bn/mix. Crisis-mode screens and 'adds 0 tasks' not covered here</t>
+        </is>
+      </c>
+      <c r="J119" s="14" t="inlineStr">
+        <is>
+          <t>tests/r5_stuck_log.test.ts</t>
+        </is>
+      </c>
       <c r="K119" s="14" t="n"/>
     </row>
     <row r="120" ht="21.75" customHeight="1" s="10">
@@ -20460,10 +20480,14 @@
       <c r="H120" s="14" t="n"/>
       <c r="I120" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J120" s="14" t="n"/>
+          <t>Partial (G1) — Automated part: focus rings, 44px targets, skip link, label and heading checks on every route in en and bn. TalkBack, 200% font on device and small-viewport device runs NOT done</t>
+        </is>
+      </c>
+      <c r="J120" s="14" t="inlineStr">
+        <is>
+          <t>tests/a11y.test.ts</t>
+        </is>
+      </c>
       <c r="K120" s="14" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1" s="10">
@@ -21797,10 +21821,14 @@
       <c r="H149" s="14" t="n"/>
       <c r="I149" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J149" s="14" t="n"/>
+          <t>Partial (G1) — Research contract via Wikipedia provider: 2-3 options with source and date, HTTP error never crashes, saved term read first. UI select/compare/reject/defer actions not covered; research contract: 0 calls without click, &lt;2 results invents nothing (unit)</t>
+        </is>
+      </c>
+      <c r="J149" s="14" t="inlineStr">
+        <is>
+          <t>tests/wikipedia.test.ts; tests/research.test.ts</t>
+        </is>
+      </c>
       <c r="K149" s="14" t="n"/>
     </row>
     <row r="150" ht="21.75" customHeight="1" s="10">
@@ -21887,10 +21915,14 @@
       <c r="H151" s="14" t="n"/>
       <c r="I151" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J151" s="14" t="n"/>
+          <t>Partial (G1) — Habits: two missed days gives a kind restart offer, never red or run-count copy; no run-count or score function. Cue/frequency/goal link not covered</t>
+        </is>
+      </c>
+      <c r="J151" s="14" t="inlineStr">
+        <is>
+          <t>tests/focus_habits_cards_ui.test.ts; tests/focus_habits_cards.test.ts</t>
+        </is>
+      </c>
       <c r="K151" s="14" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1" s="10">
@@ -22022,10 +22054,14 @@
       <c r="H154" s="14" t="n"/>
       <c r="I154" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J154" s="14" t="n"/>
+          <t>Partial (G1) — Sensitive topics (emotions, health, money, deen) carry a sensitive flag; app links are real routes. Advice-boundary note and expert-review flag on each finance/legal/tax/medical/religious screen NOT covered</t>
+        </is>
+      </c>
+      <c r="J154" s="14" t="inlineStr">
+        <is>
+          <t>tests/topics_rewards.test.ts</t>
+        </is>
+      </c>
       <c r="K154" s="14" t="n"/>
     </row>
     <row r="155" ht="15" customHeight="1" s="10">
@@ -22206,10 +22242,14 @@
       </c>
       <c r="I158" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J158" s="14" t="n"/>
+          <t>Partial (G1) — Lock-screen text hidden by default for worship, health, money and third-party; per-category 'Show details' opt-in; neutral en/bn/mix text. On-device lock-screen check, app lock and passphrase recovery NOT done (Owner)</t>
+        </is>
+      </c>
+      <c r="J158" s="14" t="inlineStr">
+        <is>
+          <t>src/core/notify.ts; tests/o8_notify_privacy.test.ts; tests/notify.test.ts</t>
+        </is>
+      </c>
       <c r="K158" s="14" t="n"/>
     </row>
     <row r="159" ht="21.75" customHeight="1" s="10">
@@ -22345,10 +22385,14 @@
       <c r="H161" s="14" t="n"/>
       <c r="I161" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J161" s="14" t="n"/>
+          <t>Partial (G1) — Horizon view places goals from stored data; unset goals kept apart; empty horizons are empty, not zero. Gantt, kanban, resource and readiness maps and text-equivalent check NOT covered</t>
+        </is>
+      </c>
+      <c r="J161" s="14" t="inlineStr">
+        <is>
+          <t>tests/horizon.test.ts</t>
+        </is>
+      </c>
       <c r="K161" s="14" t="n"/>
     </row>
     <row r="162" ht="21.75" customHeight="1" s="10">
@@ -22484,12 +22528,12 @@
       <c r="H164" s="14" t="n"/>
       <c r="I164" s="14" t="inlineStr">
         <is>
-          <t>Partial (G1) — Bangla glossary (30 terms) + field help exist. Human reviewer sign-off NOT done</t>
+          <t>Partial (G1) — Bangla glossary (30 terms) + field help exist. Human reviewer sign-off NOT done; every key present and non-empty in en, bn and mix (unit parity)</t>
         </is>
       </c>
       <c r="J164" s="14" t="inlineStr">
         <is>
-          <t>src/catalog/glossary.ts</t>
+          <t>src/catalog/glossary.ts; tests/i18n_modes.test.ts</t>
         </is>
       </c>
       <c r="K164" s="14" t="n"/>
@@ -22672,10 +22716,14 @@
       <c r="H168" s="14" t="n"/>
       <c r="I168" s="14" t="inlineStr">
         <is>
-          <t>Not run — specification stage</t>
-        </is>
-      </c>
-      <c r="J168" s="14" t="n"/>
+          <t>Partial (G1) — O5 scoring and path fit keep unknown as unknown (not_enough_data, no guess, no 0). 'incomplete' label on early path suggestions and the full assessment flow not covered</t>
+        </is>
+      </c>
+      <c r="J168" s="14" t="inlineStr">
+        <is>
+          <t>tests/o5_assessment_fit.test.ts</t>
+        </is>
+      </c>
       <c r="K168" s="14" t="n"/>
     </row>
     <row r="169" ht="21.75" customHeight="1" s="10">

</xml_diff>